<commit_message>
Privacidad de costos en catalogo publico, ajuste estricto de garantias en cotizaciones y detalles completos de Memoria RAM MTS-0057
</commit_message>
<xml_diff>
--- a/inventario_max_technology_store.xlsx
+++ b/inventario_max_technology_store.xlsx
@@ -6919,18 +6919,34 @@
       </c>
       <c r="B60" s="53" t="inlineStr">
         <is>
-          <t>Memoria Ddr4 8gb 2400t Samsung Portatil</t>
-        </is>
-      </c>
-      <c r="C60" s="54" t="inlineStr"/>
+          <t>Memoria RAM Samsung 8GB DDR4 2400MHz SODIMM para Portátil (PC4-2400T)</t>
+        </is>
+      </c>
+      <c r="C60" s="54" t="inlineStr">
+        <is>
+          <t>Almacenamiento y Memorias</t>
+        </is>
+      </c>
       <c r="D60" s="54" t="inlineStr">
         <is>
           <t>Samsung</t>
         </is>
       </c>
-      <c r="E60" s="55" t="inlineStr"/>
-      <c r="F60" s="55" t="inlineStr"/>
-      <c r="G60" s="55" t="inlineStr"/>
+      <c r="E60" s="55" t="inlineStr">
+        <is>
+          <t>M471A1K43CB1-CRC</t>
+        </is>
+      </c>
+      <c r="F60" s="55" t="inlineStr">
+        <is>
+          <t>Verde</t>
+        </is>
+      </c>
+      <c r="G60" s="55" t="inlineStr">
+        <is>
+          <t>Sin código</t>
+        </is>
+      </c>
       <c r="H60" s="55" t="inlineStr">
         <is>
           <t>REMANUFACTURADO</t>
@@ -6983,7 +6999,7 @@
       </c>
       <c r="U60" s="55" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Sin garantía</t>
         </is>
       </c>
       <c r="V60" s="54" t="inlineStr">
@@ -6991,8 +7007,22 @@
           <t>IMAGENES DE PRODUCTOS/DDR4_8GB_2400MHZ.webp</t>
         </is>
       </c>
-      <c r="W60" s="54" t="inlineStr"/>
-      <c r="X60" s="54" t="inlineStr"/>
+      <c r="W60" s="54" t="inlineStr">
+        <is>
+          <t>• Capacidad: 8 GB
+• Tipo: Memoria RAM DDR4 SODIMM para computadores portátiles / laptops
+• Frecuencia / Velocidad: 2400 MHz (PC4-2400T)
+• Formato: 260 pines SODIMM
+• Voltaje: 1.2V
+• Latencia: CL17
+• Ideal para repotenciar y acelerar portátiles de diversas marcas (HP, Lenovo, Dell, Asus, Acer).</t>
+        </is>
+      </c>
+      <c r="X60" s="54" t="inlineStr">
+        <is>
+          <t>100% testeada con MemTest86 en taller.</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="63" t="n"/>

</xml_diff>

<commit_message>
Actualización desde Panel Admin Local
</commit_message>
<xml_diff>
--- a/inventario_max_technology_store.xlsx
+++ b/inventario_max_technology_store.xlsx
@@ -5825,10 +5825,10 @@
         </is>
       </c>
       <c r="J49" s="58" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K49" s="59" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L49" s="55" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Ingreso de nuevos productos: Monitores Dahua 27 144Hz (10u), SSD M.2 ADATA Legend 710 1TB (2u) y Teclado Acer Aspire (1u) con sincronizacion a Excel y catalogo web
</commit_message>
<xml_diff>
--- a/inventario_max_technology_store.xlsx
+++ b/inventario_max_technology_store.xlsx
@@ -4912,7 +4912,7 @@
       </c>
       <c r="B40" s="53" t="inlineStr">
         <is>
-          <t>Monitor Dahua 27" Panel IPS 144Hz 1ms Full HD</t>
+          <t>Monitor Dahua LED 27 Pulgadas FHD 144Hz 1ms IPS (DHI-LM27-A221Y)</t>
         </is>
       </c>
       <c r="C40" s="54" t="inlineStr">
@@ -4930,7 +4930,11 @@
           <t>DHI-LM27-A221Y</t>
         </is>
       </c>
-      <c r="F40" s="55" t="inlineStr"/>
+      <c r="F40" s="55" t="inlineStr">
+        <is>
+          <t>Negro</t>
+        </is>
+      </c>
       <c r="G40" s="56" t="inlineStr">
         <is>
           <t>6938596001279</t>
@@ -4938,30 +4942,30 @@
       </c>
       <c r="H40" s="55" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="I40" s="57" t="inlineStr">
         <is>
-          <t>⚪ Agotado</t>
+          <t>🟢 En Stock</t>
         </is>
       </c>
       <c r="J40" s="58" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K40" s="59" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="L40" s="55" t="inlineStr">
         <is>
-          <t>Estante B - Nivel 1</t>
+          <t>Bodega / Taller - Estante Monitores</t>
         </is>
       </c>
       <c r="M40" s="60" t="n">
-        <v>327513</v>
+        <v>311071</v>
       </c>
       <c r="N40" s="61" t="n">
-        <v>0.25</v>
+        <v>0.20238</v>
       </c>
       <c r="O40" s="62">
         <f>IF(N40&lt;1, ROUNDUP(M40/(1-N40), -3), M40)</f>
@@ -4993,17 +4997,23 @@
       </c>
       <c r="V40" s="54" t="inlineStr">
         <is>
-          <t>identidad visual max tech/Logo MAX Tech.png</t>
+          <t>IMAGENES DE PRODUCTOS/Monitor dahua led 27 pulgadas ips 144 hz full hd.webp</t>
         </is>
       </c>
       <c r="W40" s="54" t="inlineStr">
         <is>
-          <t>Monitor grande de 27 pulgadas Full HD con panel IPS a 144Hz. Brinda un espacio de trabajo amplio y descansado para tener varias ventanas abiertas al tiempo, ver videos o jugar con máxima fluidez. Tiene marco ultradelgado, puertos HDMI y VGA, y 3 años de garantía.</t>
+          <t>• Pantalla: 27 Pulgadas Full HD (1920 x 1080) antirreflejo
+• Panel: IPS con ángulos de visión amplios de 178°
+• Tasa de refresco: 144 Hz ultrarrápida
+• Tiempo de respuesta: 1 ms
+• Conectividad: Puertos HDMI y VGA
+• Diseño: Biseles ultradelgados con base plástica resistente
+• Garantía oficial de 3 años Dahua.</t>
         </is>
       </c>
       <c r="X40" s="54" t="inlineStr">
         <is>
-          <t>Gran formato de 27 pulgadas.</t>
+          <t>10 unidades físicas selladas. Seriales: BLR01916302500002 a BLR01916302500646. Factura FT-9364.</t>
         </is>
       </c>
     </row>
@@ -7342,8 +7352,229 @@
       <c r="W63" s="68" t="inlineStr"/>
       <c r="X63" s="68" t="inlineStr"/>
     </row>
-    <row r="64"/>
-    <row r="65"/>
+    <row r="64">
+      <c r="A64" s="77" t="inlineStr">
+        <is>
+          <t>MTS-0061</t>
+        </is>
+      </c>
+      <c r="B64" s="67" t="inlineStr">
+        <is>
+          <t>Disco Estado Sólido SSD M.2 NVMe 1TB ADATA Legend 710 PCIe Gen3 x4</t>
+        </is>
+      </c>
+      <c r="C64" s="68" t="inlineStr">
+        <is>
+          <t>Almacenamiento y Memorias</t>
+        </is>
+      </c>
+      <c r="D64" s="68" t="inlineStr">
+        <is>
+          <t>ADATA</t>
+        </is>
+      </c>
+      <c r="E64" s="69" t="inlineStr">
+        <is>
+          <t>ALEG-710-1TCS</t>
+        </is>
+      </c>
+      <c r="F64" s="69" t="inlineStr">
+        <is>
+          <t>Azul / Negro</t>
+        </is>
+      </c>
+      <c r="G64" s="69" t="inlineStr">
+        <is>
+          <t>4711085635398</t>
+        </is>
+      </c>
+      <c r="H64" s="69" t="inlineStr">
+        <is>
+          <t>NUEVO</t>
+        </is>
+      </c>
+      <c r="I64" s="70" t="inlineStr">
+        <is>
+          <t>🟢 En Stock</t>
+        </is>
+      </c>
+      <c r="J64" s="70" t="n">
+        <v>2</v>
+      </c>
+      <c r="K64" s="69" t="n">
+        <v>2</v>
+      </c>
+      <c r="L64" s="69" t="inlineStr">
+        <is>
+          <t>Vitrina Accesorios / Taller</t>
+        </is>
+      </c>
+      <c r="M64" s="78" t="n">
+        <v>530000</v>
+      </c>
+      <c r="N64" s="79" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O64" s="80">
+        <f>IF(N64&lt;1, ROUNDUP(M64/(1-N64), -3), M64)</f>
+        <v/>
+      </c>
+      <c r="P64" s="79" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="Q64" s="78">
+        <f>IF((1-N64-P64)&gt;0, ROUNDUP((M64+IF(O64&gt;=90000,20000,0))/(1-N64-P64), -3), O64)</f>
+        <v/>
+      </c>
+      <c r="R64" s="78">
+        <f>O64</f>
+        <v/>
+      </c>
+      <c r="S64" s="78">
+        <f>O64-M64</f>
+        <v/>
+      </c>
+      <c r="T64" s="79">
+        <f>IF(O64&gt;0, (O64-M64)/O64, 0)</f>
+        <v/>
+      </c>
+      <c r="U64" s="69" t="inlineStr">
+        <is>
+          <t>6 Meses</t>
+        </is>
+      </c>
+      <c r="V64" s="68" t="inlineStr">
+        <is>
+          <t>IMAGENES DE PRODUCTOS/ADATA_LEGEND_710_1TB.jpg</t>
+        </is>
+      </c>
+      <c r="W64" s="68" t="inlineStr">
+        <is>
+          <t>• Capacidad: 1 TB (1000 GB)
+• Formato: M.2 2280
+• Interfaz: PCIe Gen3 x4 NVMe 1.4
+• Velocidad de lectura secuencial: Hasta 2.400 MB/s
+• Velocidad de escritura secuencial: Hasta 1.800 MB/s
+• Disipador térmico de aluminio incluido (reduce temperatura hasta 15%)
+• Compatible con PCs de escritorio y portátiles con slot M.2 NVMe.</t>
+        </is>
+      </c>
+      <c r="X64" s="68" t="inlineStr">
+        <is>
+          <t>2 unidades físicas. Seriales: 4P2220413136, 4P2220410141. Facturas FEVO 33176 y 33181.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="77" t="inlineStr">
+        <is>
+          <t>MTS-0062</t>
+        </is>
+      </c>
+      <c r="B65" s="67" t="inlineStr">
+        <is>
+          <t>Teclado para Portátil Acer Aspire E1-470 E5-471P V3-472 3830T 4830 Negro Español</t>
+        </is>
+      </c>
+      <c r="C65" s="68" t="inlineStr">
+        <is>
+          <t>Periféricos y Accesorios</t>
+        </is>
+      </c>
+      <c r="D65" s="68" t="inlineStr">
+        <is>
+          <t>Acer / Compatible</t>
+        </is>
+      </c>
+      <c r="E65" s="69" t="inlineStr">
+        <is>
+          <t>00002272</t>
+        </is>
+      </c>
+      <c r="F65" s="69" t="inlineStr">
+        <is>
+          <t>Negro</t>
+        </is>
+      </c>
+      <c r="G65" s="69" t="inlineStr">
+        <is>
+          <t>Sin código</t>
+        </is>
+      </c>
+      <c r="H65" s="69" t="inlineStr">
+        <is>
+          <t>NUEVO</t>
+        </is>
+      </c>
+      <c r="I65" s="70" t="inlineStr">
+        <is>
+          <t>🟢 En Stock</t>
+        </is>
+      </c>
+      <c r="J65" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="K65" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="L65" s="69" t="inlineStr">
+        <is>
+          <t>Taller - Repuestos</t>
+        </is>
+      </c>
+      <c r="M65" s="78" t="n">
+        <v>50000</v>
+      </c>
+      <c r="N65" s="79" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="O65" s="80">
+        <f>IF(N65&lt;1, ROUNDUP(M65/(1-N65), -3), M65)</f>
+        <v/>
+      </c>
+      <c r="P65" s="79" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="Q65" s="78">
+        <f>IF((1-N65-P65)&gt;0, ROUNDUP((M65+IF(O65&gt;=90000,20000,0))/(1-N65-P65), -3), O65)</f>
+        <v/>
+      </c>
+      <c r="R65" s="78">
+        <f>O65</f>
+        <v/>
+      </c>
+      <c r="S65" s="78">
+        <f>O65-M65</f>
+        <v/>
+      </c>
+      <c r="T65" s="79">
+        <f>IF(O65&gt;0, (O65-M65)/O65, 0)</f>
+        <v/>
+      </c>
+      <c r="U65" s="69" t="inlineStr">
+        <is>
+          <t>6 Meses</t>
+        </is>
+      </c>
+      <c r="V65" s="68" t="inlineStr">
+        <is>
+          <t>identidad visual max tech/Logo MAX Tech.png</t>
+        </is>
+      </c>
+      <c r="W65" s="68" t="inlineStr">
+        <is>
+          <t>• Idioma / Distribución: Español con letra Ñ
+• Color: Negro mate
+• Compatibilidad: Acer Aspire E1-470, E1-470G, E1-472, E5-471, E5-471P, V3-472, 3830, 3830T, 4830, 4830T
+• Tipo de repuesto: Teclado de reemplazo de alta respuesta táctil.</t>
+        </is>
+      </c>
+      <c r="X65" s="68" t="inlineStr">
+        <is>
+          <t>Serial: 2F50031050103. Factura FEVO 33009.</t>
+        </is>
+      </c>
+    </row>
     <row r="66"/>
     <row r="67"/>
     <row r="68"/>

</xml_diff>